<commit_message>
Use an authorized real collection record in the layout sampler
</commit_message>
<xml_diff>
--- a/examples/label_options_examples.xlsx
+++ b/examples/label_options_examples.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -514,7 +514,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEMO000001</t>
+          <t>BBSL1207977</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -534,17 +534,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Example Meadow</t>
+          <t>Tony Grove, 0.5km NNE</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>41.9</v>
+        <v>41.89971</v>
       </c>
       <c r="G2" t="n">
-        <v>-111.65</v>
+        <v>-111.64205</v>
       </c>
       <c r="H2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -553,159 +553,27 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>12Jul2026</t>
+          <t>24Jun2022</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>A. Smith</t>
+          <t>M. Branstetter, C. Meidt</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>meadow</t>
+          <t>alpine meadow</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>pan traps</t>
+          <t>Taraxacum officinale</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>EVT001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DEMO000002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Cache Co.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Example Meadow</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-111.65</v>
-      </c>
-      <c r="H3" t="n">
-        <v>100</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2500m</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>12Jul2026</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>A. Smith, B. Jones</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>meadow</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Phacelia sp.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>EVT001</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DEMO000003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Cache Co.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Example Ridge</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>41.91</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-111.66</v>
-      </c>
-      <c r="H4" t="n">
-        <v>500</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2800m</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>13Jul2026</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>A. Smith</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>rocky alpine woodland</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Phacelia tanacetifolia</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>EVT002</t>
+          <t>MGB4209</t>
         </is>
       </c>
     </row>
@@ -720,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -814,7 +682,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEMO000001</t>
+          <t>BBSL1207977</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -834,17 +702,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Example Meadow</t>
+          <t>Tony Grove, 0.5km NNE</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>41.9</v>
+        <v>41.89971</v>
       </c>
       <c r="G2" t="n">
-        <v>-111.65</v>
+        <v>-111.64205</v>
       </c>
       <c r="H2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -853,159 +721,27 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>12Jul2026</t>
+          <t>24Jun2022</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>A. Smith</t>
+          <t>M. Branstetter, C. Meidt</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>meadow</t>
+          <t>alpine meadow</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>pan traps</t>
+          <t>Taraxacum officinale</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>EVT001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DEMO000002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Cache Co.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Example Meadow</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-111.65</v>
-      </c>
-      <c r="H3" t="n">
-        <v>100</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2500m</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>12Jul2026</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>A. Smith, B. Jones</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>meadow</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Phacelia sp.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>EVT001</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DEMO000003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Cache Co.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Example Ridge</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>41.91</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-111.66</v>
-      </c>
-      <c r="H4" t="n">
-        <v>500</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2800m</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>13Jul2026</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>A. Smith</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>rocky alpine woodland</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Phacelia tanacetifolia</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>EVT002</t>
+          <t>MGB4209</t>
         </is>
       </c>
     </row>
@@ -1020,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1114,7 +850,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEMO000001</t>
+          <t>BBSL1207977</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1134,17 +870,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Example Meadow</t>
+          <t>Tony Grove, 0.5km NNE</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>41.9</v>
+        <v>41.89971</v>
       </c>
       <c r="G2" t="n">
-        <v>-111.65</v>
+        <v>-111.64205</v>
       </c>
       <c r="H2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1153,159 +889,27 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>12Jul2026</t>
+          <t>24Jun2022</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>A. Smith</t>
+          <t>M. Branstetter, C. Meidt</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>meadow</t>
+          <t>alpine meadow</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>pan traps</t>
+          <t>Taraxacum officinale</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>EVT001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DEMO000002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Cache Co.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Example Meadow</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-111.65</v>
-      </c>
-      <c r="H3" t="n">
-        <v>100</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2500m</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>12Jul2026</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>A. Smith, B. Jones</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>meadow</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Phacelia sp.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>EVT001</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DEMO000003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Cache Co.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Example Ridge</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>41.91</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-111.66</v>
-      </c>
-      <c r="H4" t="n">
-        <v>500</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2800m</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>13Jul2026</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>A. Smith</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>rocky alpine woodland</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Phacelia tanacetifolia</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>EVT002</t>
+          <t>MGB4209</t>
         </is>
       </c>
     </row>
@@ -1320,7 +924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1420,7 +1024,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEMO000001</t>
+          <t>BBSL1207977</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1440,17 +1044,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Example Meadow</t>
+          <t>Tony Grove, 0.5km NNE</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>41.9</v>
+        <v>41.89971</v>
       </c>
       <c r="G2" t="n">
-        <v>-111.65</v>
+        <v>-111.64205</v>
       </c>
       <c r="H2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -1459,172 +1063,30 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>12Jul2026</t>
+          <t>24Jun2022</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>A. Smith</t>
+          <t>M. Branstetter, C. Meidt</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>meadow</t>
+          <t>alpine meadow</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Phacelia sp.</t>
+          <t>Taraxacum officinale</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>EVT001</t>
+          <t>MGB4209</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
-        <is>
-          <t>net</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DEMO000002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Cache Co.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Example Meadow</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-111.65</v>
-      </c>
-      <c r="H3" t="n">
-        <v>100</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2500m</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>12Jul2026</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>A. Smith, B. Jones</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>meadow</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Phacelia sp.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>EVT001</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>net</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DEMO000003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>UT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Cache Co.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Example Ridge</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>41.91</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-111.66</v>
-      </c>
-      <c r="H4" t="n">
-        <v>500</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2800m</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>13Jul2026</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>A. Smith</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>meadow</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Phacelia sp.</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>EVT002</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
         <is>
           <t>net</t>
         </is>
@@ -1641,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1657,21 +1119,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEMO000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DEMO000002</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DEMO000003</t>
+          <t>BBSL1207977</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1826,21 +1274,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEMO000001</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DEMO000002</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DEMO000003</t>
+          <t>BBSL1207977</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1958,6 +1392,18 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Example provenance</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BBSL1207977 / MGB4209: real collection data, shared with permission. Determination remains fictional; no identification supplied.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add compact five-line collection labels without barcodes
</commit_message>
<xml_diff>
--- a/examples/label_options_examples.xlsx
+++ b/examples/label_options_examples.xlsx
@@ -15,6 +15,8 @@
     <sheet name="Determination" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Pin_Barcode" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Instructions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Collection_Only" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Collection_Only_Paired" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -582,6 +584,174 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>StateProvince</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>LocalityLabel</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Uncertainty</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Verbatim_Elevation</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Verbatim_Date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Collector_Label</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>MacroHabitat_Label</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Microhabitat_Label</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Field_Number</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Sampling_Protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cache Co.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Tony Grove, 0.5km NNE</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>41.89971</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-111.64205</v>
+      </c>
+      <c r="G2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2500m</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>24Jun2022</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>M. Branstetter, C. Meidt</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>alpine meadow</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Taraxacum officinale</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>MGB4209</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>net</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1289,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1404,6 +1574,187 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Collection_Only</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>--mode collection-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Collection_Only_Paired</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>--mode collection-only --separate-habitat --include-method</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>StateProvince</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>LocalityLabel</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Uncertainty</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Verbatim_Elevation</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Verbatim_Date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Collector_Label</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>MacroHabitat_Label</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Microhabitat_Label</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Field_Number</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cache Co.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Tony Grove, 0.5km NNE</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>41.89971</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-111.64205</v>
+      </c>
+      <c r="G2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2500m</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>24Jun2022</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>M. Branstetter, C. Meidt</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>alpine meadow</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Taraxacum officinale</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>MGB4209</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add wrapped single collection-only labels
</commit_message>
<xml_diff>
--- a/examples/label_options_examples.xlsx
+++ b/examples/label_options_examples.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Instructions" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Collection_Only" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Collection_Only_Paired" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Collection_Only_Wrapped" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -752,6 +753,163 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>StateProvince</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>LocalityLabel</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Uncertainty</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Verbatim_Elevation</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Verbatim_Date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Collector_Label</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>MacroHabitat_Label</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Microhabitat_Label</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Field_Number</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cache Co.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Tony Grove, 0.5km NNE</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>41.89971</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-111.64205</v>
+      </c>
+      <c r="G2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2500m</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>24Jun2022</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>M. Branstetter, C. Meidt</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>alpine meadow</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Taraxacum officinale</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>MGB4209</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1459,7 +1617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1595,6 +1753,18 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>--mode collection-only --separate-habitat --include-method</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Collection_Only_Wrapped</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>--mode collection-only --layout flow</t>
         </is>
       </c>
     </row>

</xml_diff>